<commit_message>
Sheet 00: ⟦INVENTORY⟧ — every dataset 01 … 11
The register in sheet 00 lists what a pack carries, so a dataset missing from it
might be absent from the treaty or might never have been specified at all. The
new ⟦INVENTORY⟧ block tells the two apart: role, sheet, what it holds, and what
state it is in. Written into all seven reference packs from one shared table, so
they cannot drift.

Exchange rates is numbered 11. It was the one sheet without a number, which made
it the one sheet §2.2's ordering could not place.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgDs1kQm7zUEUCoe8K4YPd
</commit_message>
<xml_diff>
--- a/Intake_EngineeringCombined_v1.xlsx
+++ b/Intake_EngineeringCombined_v1.xlsx
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +136,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -518,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:V98"/>
+  <dimension ref="B1:V115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -971,1047 +972,1347 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>⟦SECTIONS⟧</t>
+          <t>⟦INVENTORY⟧</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Kind</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Datasets</t>
+          <t>Holds</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>State</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>per risk</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>History</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>01, 02, 03, 04, 05</t>
+          <t>Premium and loss history per section</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>EPI Projections</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Estimated premium income, N and N+1</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>A section is a block. Per-risk sections carry large losses (03); cat sections carry event losses (04) instead. Rules are scoped by kind and evaluated once per applicable section, so an absent dataset is 'not applicable', not a gap.</t>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Large Losses</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Individual large claims, per-risk sections</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Cat Losses</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Catastrophe events, cat sections</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>⟦GLOBAL⟧</t>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Risk Profiles</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Banded exposure — the per-risk rating basis</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Value</t>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>EQ Aggs</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Earthquake sums insured per cat zone</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Actual year</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>2025</v>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Wind Aggs</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Windstorm sums insured per cat zone</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>implemented</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Treaty type</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Engineering</t>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Splits</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Occupancy x cover (Fire) or x Projects/Renewables (Eng.)</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>axes settled, measures open</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Cedent</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Example Insurance SA</t>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Rate Development</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Rate change history — optional</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>outstanding</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Loss share warning</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="n">
-        <v>0.2</v>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Triangles</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Loss development triangles</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>outstanding</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Exchange rates</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>FX rates for conversion between currencies</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>outstanding</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Actual year is N: the expiring year; the renewal is N+1. Sheet attributes override these; block attributes override the sheet. Loss share warning is the point above which a year's declared losses are flagged (§10.3).</t>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Collected step-2 blocks — written, never read</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>outstanding</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>⟦TYPES⟧</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Type</t>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Every dataset the tool knows, whether or not this pack carries it. The register above lists what is here; ⟦SECTIONS⟧ says which roles each section expects, so a missing sheet reads as structure rather than as a gap.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>⟦SECTIONS⟧</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Datasets</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Incurred Losses</t>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>number</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>EPI</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+          <t>per risk</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>01, 02, 03, 04, 05</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Band</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Band from</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>A section is a block. Per-risk sections carry large losses (03); cat sections carry event losses (04) instead. Rules are scoped by kind and evaluated once per applicable section, so an absent dataset is 'not applicable', not a gap.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Band to</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>⟦GLOBAL⟧</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Number of Risks</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Exposure</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
+          <t>Actual year</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>2025</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Claim Reference</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
+          <t>Treaty type</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Name of Loss</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
+          <t>Cedent</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Example Insurance SA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Event ID</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
+          <t>Loss share warning</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Loss amount</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Number of Claims</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>number</t>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Actual year is N: the expiring year; the renewal is N+1. Sheet attributes override these; block attributes override the sheet. Loss share warning is the point above which a year's declared losses are flagged (§10.3).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Date of Loss</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>date</t>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>⟦TYPES⟧</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Event Date</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>date</t>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Event End Date</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>A field name carries one type across the whole workbook.</t>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Incurred Losses</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>EPI</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>⟦VOCABULARY⟧</t>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Permitted values</t>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Band from</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Year basis</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>UW | Occurrence</t>
+          <t>Band to</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Premium basis</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>GWP | GNPI | Written | Earned | Signed</t>
+          <t>Number of Risks</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Loss basis</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Paid | Incurred</t>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>PF transfer</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>with clean cut | without clean cut | none</t>
+          <t>Claim Reference</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Exposure basis</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Sum Insured | EML | PML | MPL</t>
+          <t>Name of Loss</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Includes fac</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>yes | no</t>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Layered business</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>included | excluded</t>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Scale</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>1 | 1,000 | 1,000,000</t>
+          <t>Loss amount</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Share basis</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>100% | ceded only</t>
+          <t>Number of Claims</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Date format</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>ISO | DD.MM.YYYY | MM/DD/YYYY</t>
+          <t>Date of Loss</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Occurrence year from</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Event Date | Event End Date</t>
+          <t>Event Date</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="4" t="inlineStr">
         <is>
+          <t>Event End Date</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>A field name carries one type across the whole workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>⟦VOCABULARY⟧</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Permitted values</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Year basis</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>UW | Occurrence</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Premium basis</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>GWP | GNPI | Written | Earned | Signed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Loss basis</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Paid | Incurred</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>PF transfer</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>with clean cut | without clean cut | none</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Exposure basis</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Sum Insured | EML | PML | MPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Includes fac</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>yes | no</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Layered business</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>included | excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>1 | 1,000 | 1,000,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Share basis</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>100% | ceded only</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Date format</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>ISO | DD.MM.YYYY | MM/DD/YYYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Occurrence year from</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Event Date | Event End Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="4" t="inlineStr">
+        <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>ISO 4217</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" s="3" t="inlineStr">
+    <row r="83">
+      <c r="B83" s="3" t="inlineStr">
         <is>
           <t>⟦PERIOD ORDER⟧</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" s="7" t="inlineStr">
+    <row r="84">
+      <c r="B84" s="7" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="C67" s="7" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr">
         <is>
           <t>Suffix</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" s="10" t="n">
+    <row r="85">
+      <c r="B85" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>est</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="10" t="n">
+    <row r="86">
+      <c r="B86" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>9 months</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" s="10" t="n">
+    <row r="87">
+      <c r="B87" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C87" s="5" t="inlineStr">
         <is>
           <t>re-est</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" s="2" t="inlineStr">
+    <row r="89">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>Within one year the suffixes sort in this order, not alphabetically. A bare year sorts first; an unlisted suffix sorts last.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="B74" s="3" t="inlineStr">
+    <row r="91">
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>⟦RULES⟧</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="B75" s="7" t="inlineStr">
+    <row r="92">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>Left</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Rel</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="E92" s="7" t="inlineStr">
         <is>
           <t>Right</t>
         </is>
       </c>
-      <c r="F75" s="7" t="inlineStr">
+      <c r="F92" s="7" t="inlineStr">
         <is>
           <t>Tolerance</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G92" s="7" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="H92" s="7" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="I75" s="7" t="inlineStr">
+      <c r="I92" s="7" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" s="7" t="inlineStr">
+    <row r="93">
+      <c r="B93" s="7" t="inlineStr">
         <is>
           <t>R-05</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C93" s="12" t="inlineStr">
         <is>
           <t>01.Premium@{N} 9 months</t>
         </is>
       </c>
-      <c r="D76" s="7" t="inlineStr">
+      <c r="D93" s="7" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E76" s="11" t="inlineStr">
+      <c r="E93" s="12" t="inlineStr">
         <is>
           <t>02.EPI@{N} 9 months</t>
         </is>
       </c>
-      <c r="F76" s="4" t="n">
+      <c r="F93" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G76" s="4" t="inlineStr">
+      <c r="G93" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="H76" s="5" t="inlineStr">
+      <c r="H93" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="I93" s="2" t="inlineStr">
         <is>
           <t>same nine months reported in two sheets</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="B77" s="7" t="inlineStr">
+    <row r="94">
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>R-06</t>
         </is>
       </c>
-      <c r="C77" s="11" t="inlineStr">
+      <c r="C94" s="12" t="inlineStr">
         <is>
           <t>01.Premium@{N}</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E77" s="11" t="inlineStr">
+      <c r="E94" s="12" t="inlineStr">
         <is>
           <t>02.EPI@{N} re-est</t>
         </is>
       </c>
-      <c r="F77" s="4" t="n">
+      <c r="F94" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G77" s="4" t="inlineStr">
+      <c r="G94" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="H77" s="5" t="inlineStr">
+      <c r="H94" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="I94" s="2" t="inlineStr">
         <is>
           <t>a full-year N in History is an estimate, not an actual</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="B78" s="7" t="inlineStr">
+    <row r="95">
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>R-07</t>
         </is>
       </c>
-      <c r="C78" s="11" t="inlineStr">
+      <c r="C95" s="12" t="inlineStr">
         <is>
           <t>02.EPI@{N} re-est</t>
         </is>
       </c>
-      <c r="D78" s="7" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="E78" s="11" t="inlineStr">
+      <c r="E95" s="12" t="inlineStr">
         <is>
           <t>02.EPI@{N} 9 months</t>
         </is>
       </c>
-      <c r="F78" s="4" t="n">
+      <c r="F95" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G78" s="4" t="inlineStr">
+      <c r="G95" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="H78" s="5" t="inlineStr">
+      <c r="H95" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="I95" s="2" t="inlineStr">
         <is>
           <t>premium accrues; a re-estimate cannot fall below what is booked</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="B79" s="7" t="inlineStr">
+    <row r="96">
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>R-01</t>
         </is>
       </c>
-      <c r="C79" s="11" t="inlineStr">
+      <c r="C96" s="12" t="inlineStr">
         <is>
           <t>SUM(03.Loss amount@{Y})</t>
         </is>
       </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E79" s="11" t="inlineStr">
+      <c r="E96" s="12" t="inlineStr">
         <is>
           <t>01.Incurred Losses@{Y}</t>
         </is>
       </c>
-      <c r="F79" s="4" t="n">
+      <c r="F96" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="4" t="inlineStr">
+      <c r="G96" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="H79" s="5" t="inlineStr">
+      <c r="H96" s="5" t="inlineStr">
         <is>
           <t>per risk</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>large losses cannot exceed total incurred for the same year</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="B80" s="7" t="inlineStr">
+    <row r="97">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>R-02</t>
         </is>
       </c>
-      <c r="C80" s="11" t="inlineStr">
+      <c r="C97" s="12" t="inlineStr">
         <is>
           <t>SUM(04.Loss amount@{Y})</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E80" s="11" t="inlineStr">
+      <c r="E97" s="12" t="inlineStr">
         <is>
           <t>01.Incurred Losses@{Y}</t>
         </is>
       </c>
-      <c r="F80" s="4" t="n">
+      <c r="F97" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="G97" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr">
+      <c r="H97" s="5" t="inlineStr">
         <is>
           <t>cat</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="I97" s="2" t="inlineStr">
         <is>
           <t>cat losses cannot exceed total incurred for the same year</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" s="7" t="inlineStr">
-        <is>
-          <t>R-09</t>
-        </is>
-      </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>01.Year basis</t>
-        </is>
-      </c>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="E81" s="11" t="inlineStr">
-        <is>
-          <t>03.Year basis</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H81" s="5" t="inlineStr">
-        <is>
-          <t>per risk</t>
-        </is>
-      </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>history and large losses must be on the same year basis</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="7" t="inlineStr">
-        <is>
-          <t>R-10</t>
-        </is>
-      </c>
-      <c r="C82" s="11" t="inlineStr">
-        <is>
-          <t>01.Year basis</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="E82" s="11" t="inlineStr">
-        <is>
-          <t>04.Year basis</t>
-        </is>
-      </c>
-      <c r="F82" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="H82" s="5" t="inlineStr">
-        <is>
-          <t>cat</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>history and cat losses must be on the same year basis</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Forms: &lt;key or role&gt;.&lt;field&gt;@&lt;record&gt; · &lt;key&gt;.&lt;attribute&gt; · SUM(&lt;key&gt;.&lt;field&gt;@&lt;record&gt;).  {N} resolves from ⟦GLOBAL⟧; {Y} expands once per year. Scope selects the sections a rule runs over.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>⟦MARKERS⟧  —  written in column A of every other sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="7" t="inlineStr">
-        <is>
-          <t>Marker</t>
-        </is>
-      </c>
-      <c r="C87" s="7" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="12" t="inlineStr">
-        <is>
-          <t>Header_i</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>row-wise: this row is block i's extraction row (declared labels only)</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="12" t="inlineStr">
-        <is>
-          <t>Header_i = &lt;col&gt;</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>transposed: this column is block i's extraction column</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="12" t="inlineStr">
-        <is>
-          <t>Info_i = &lt;col&gt;</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>row-wise: this column holds the record selectors, =ROW()</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="12" t="inlineStr">
-        <is>
-          <t>Info_i = &lt;row&gt;</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="inlineStr">
-        <is>
-          <t>transposed: this row holds the record selectors, =COLUMN()</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="B92" s="12" t="inlineStr">
-        <is>
-          <t>Transpose_i</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>block i is transposed</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="B93" s="12" t="inlineStr">
-        <is>
-          <t>Dataset_i = &lt;key&gt;</t>
-        </is>
-      </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>which dataset block i is — defaults to the sheet-name match</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="B94" s="12" t="inlineStr">
-        <is>
-          <t>Section_i = &lt;name&gt;</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>which section of the treaty block i belongs to</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="B95" s="12" t="inlineStr">
-        <is>
-          <t>&lt;Attribute&gt; = &lt;value&gt;</t>
-        </is>
-      </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>an attribute of the sheet (unsuffixed) or block i (suffixed _i)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="12" t="inlineStr">
-        <is>
-          <t>H_&lt;Attribute&gt; = &lt;val&gt;</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>the same, declared as a hypothesis — raises a query</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>R-09</t>
+        </is>
+      </c>
+      <c r="C98" s="12" t="inlineStr">
+        <is>
+          <t>01.Year basis</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="E98" s="12" t="inlineStr">
+        <is>
+          <t>03.Year basis</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>per risk</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>history and large losses must be on the same year basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="C99" s="12" t="inlineStr">
+        <is>
+          <t>01.Year basis</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="inlineStr">
+        <is>
+          <t>04.Year basis</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>cat</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>history and cat losses must be on the same year basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Forms: &lt;key or role&gt;.&lt;field&gt;@&lt;record&gt; · &lt;key&gt;.&lt;attribute&gt; · SUM(&lt;key&gt;.&lt;field&gt;@&lt;record&gt;).  {N} resolves from ⟦GLOBAL⟧; {Y} expands once per year. Scope selects the sections a rule runs over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>⟦MARKERS⟧  —  written in column A of every other sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Marker</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="13" t="inlineStr">
+        <is>
+          <t>Header_i</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>row-wise: this row is block i's extraction row (declared labels only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="13" t="inlineStr">
+        <is>
+          <t>Header_i = &lt;col&gt;</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>transposed: this column is block i's extraction column</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="13" t="inlineStr">
+        <is>
+          <t>Info_i = &lt;col&gt;</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>row-wise: this column holds the record selectors, =ROW()</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="13" t="inlineStr">
+        <is>
+          <t>Info_i = &lt;row&gt;</t>
+        </is>
+      </c>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>transposed: this row holds the record selectors, =COLUMN()</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="13" t="inlineStr">
+        <is>
+          <t>Transpose_i</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>block i is transposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>Dataset_i = &lt;key&gt;</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>which dataset block i is — defaults to the sheet-name match</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>Section_i = &lt;name&gt;</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>which section of the treaty block i belongs to</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>&lt;Attribute&gt; = &lt;value&gt;</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>an attribute of the sheet (unsuffixed) or block i (suffixed _i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>H_&lt;Attribute&gt; = &lt;val&gt;</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>the same, declared as a hypothesis — raises a query</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="7" t="inlineStr">
         <is>
           <t>No Header_i anywhere in column A  →  nothing is extracted from that sheet.</t>
         </is>
@@ -2050,78 +2351,78 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Section = Engineering</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Currency = USD</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Scale = 1,000</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Share basis = 100%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>H_Year basis = UW</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Premium basis = GNPI</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>H_Loss basis = Incurred</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>H_PF transfer = with clean cut</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>U/W Yr</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Policies</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Prem.</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>Incurred</t>
         </is>
@@ -2133,22 +2434,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Header_1</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Incurred Losses</t>
         </is>
@@ -2160,132 +2461,132 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>410</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="19" t="n">
         <v>8200</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="19" t="n">
         <v>5100</v>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="20">
         <f>ROW()</f>
         <v>12</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>435</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <v>8640</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <v>6350</v>
       </c>
-      <c r="L13" s="19">
+      <c r="L13" s="20">
         <f>ROW()</f>
         <v>13</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>452</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="19" t="n">
         <v>9100</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <v>4820</v>
       </c>
-      <c r="L14" s="19">
+      <c r="L14" s="20">
         <f>ROW()</f>
         <v>14</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>468</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="19" t="n">
         <v>9480</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <v>7240</v>
       </c>
-      <c r="L15" s="19">
+      <c r="L15" s="20">
         <f>ROW()</f>
         <v>15</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="19" t="n">
         <v>480</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="19" t="n">
         <v>9900</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="19" t="n">
         <v>5680</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="20">
         <f>ROW()</f>
         <v>16</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Info_1 = L</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>2025 9 months</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="19" t="n">
         <v>372</v>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="19" t="n">
         <v>7420</v>
       </c>
-      <c r="G17" s="18" t="n">
+      <c r="G17" s="19" t="n">
         <v>3910</v>
       </c>
-      <c r="L17" s="19">
+      <c r="L17" s="20">
         <f>ROW()</f>
         <v>17</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>As at = 31.12.2025</t>
         </is>
@@ -2295,15 +2596,15 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="C18" s="20">
+      <c r="C18" s="21">
         <f>SUM(C12:C17)</f>
         <v>2617</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="21">
         <f>SUM(D12:D17)</f>
         <v>52740</v>
       </c>
-      <c r="G18" s="20">
+      <c r="G18" s="21">
         <f>SUM(G12:G17)</f>
         <v>33100</v>
       </c>
@@ -2344,59 +2645,59 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Section = Engineering</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Currency = USD</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Scale = 1,000</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Share basis = 100%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>H_Year basis = UW</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Premium basis = GNPI</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>EPI (net)</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Share %</t>
         </is>
@@ -2408,17 +2709,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Header_1</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>EPI</t>
         </is>
@@ -2430,75 +2731,75 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>2025 est</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="19" t="n">
         <v>9450</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="20">
         <f>ROW()</f>
         <v>11</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>2025 9 months</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>7420</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="K12" s="19">
+      <c r="K12" s="20">
         <f>ROW()</f>
         <v>12</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>2025 re-est</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>9900</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="K13" s="19">
+      <c r="K13" s="20">
         <f>ROW()</f>
         <v>13</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>10600</v>
       </c>
-      <c r="D14" s="21" t="n">
+      <c r="D14" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="K14" s="19">
+      <c r="K14" s="20">
         <f>ROW()</f>
         <v>14</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Info_1 = K</t>
         </is>
@@ -2508,7 +2809,7 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="21">
         <f>SUM(C11:C14)</f>
         <v>37370</v>
       </c>
@@ -2519,7 +2820,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>As at = 31.12.2025</t>
         </is>
@@ -2560,105 +2861,105 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Section = Engineering</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Currency = USD</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Scale = 1,000</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Share basis = 100%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>H_Year basis = UW</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>H_Loss basis = Incurred</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Date format = ISO</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Threshold = 500</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Occurrence year from = Event Date</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Claim no.</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Cat code</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>U/W Yr</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Gross incurred</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr">
+      <c r="I11" s="15" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
@@ -2670,27 +2971,27 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Header_1</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="23" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>Name of Loss</t>
         </is>
       </c>
-      <c r="F12" s="22" t="inlineStr">
+      <c r="F12" s="23" t="inlineStr">
         <is>
           <t>Loss amount</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>Date of Loss</t>
         </is>
@@ -2702,49 +3003,49 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Dataset_1 = 03 Large</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Header_2</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Event ID</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E14" s="23" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>Event Name</t>
         </is>
       </c>
-      <c r="F14" s="23" t="inlineStr">
+      <c r="F14" s="24" t="inlineStr">
         <is>
           <t>Loss amount</t>
         </is>
       </c>
-      <c r="G14" s="23" t="inlineStr">
+      <c r="G14" s="24" t="inlineStr">
         <is>
           <t>Event Date</t>
         </is>
       </c>
-      <c r="H14" s="23" t="inlineStr">
+      <c r="H14" s="24" t="inlineStr">
         <is>
           <t>Event End Date</t>
         </is>
       </c>
-      <c r="I14" s="23" t="inlineStr">
+      <c r="I14" s="24" t="inlineStr">
         <is>
           <t>Number of Claims</t>
         </is>
@@ -2756,7 +3057,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Dataset_2 = 04 Cat</t>
         </is>
@@ -2768,7 +3069,7 @@
           <t>CL-2201</t>
         </is>
       </c>
-      <c r="D16" s="17" t="inlineStr">
+      <c r="D16" s="18" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
@@ -2778,17 +3079,17 @@
           <t>Turbine erection collapse, Gdansk</t>
         </is>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>1420</v>
       </c>
-      <c r="G16" s="24" t="n">
+      <c r="G16" s="25" t="n">
         <v>44294</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="12">
         <f>IF($C16="",ROW(),"")</f>
         <v>16</v>
       </c>
-      <c r="K16" s="11" t="n"/>
+      <c r="K16" s="12" t="n"/>
     </row>
     <row r="17">
       <c r="C17" s="4" t="inlineStr">
@@ -2796,7 +3097,7 @@
           <t>EV-301</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
@@ -2806,20 +3107,20 @@
           <t>Flood, Saxony</t>
         </is>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="19" t="n">
         <v>1150</v>
       </c>
-      <c r="G17" s="24" t="n">
+      <c r="G17" s="25" t="n">
         <v>44391</v>
       </c>
-      <c r="H17" s="24" t="n">
+      <c r="H17" s="25" t="n">
         <v>44395</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11">
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12">
         <f>IF($C17&lt;&gt;"",ROW(),"")</f>
         <v>17</v>
       </c>
@@ -2830,7 +3131,7 @@
           <t>CL-2202</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
@@ -2840,17 +3141,17 @@
           <t>Tunnel boring machine damage, Oslo</t>
         </is>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <v>2310</v>
       </c>
-      <c r="G18" s="24" t="n">
+      <c r="G18" s="25" t="n">
         <v>45007</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="12">
         <f>IF($C18="",ROW(),"")</f>
         <v>18</v>
       </c>
-      <c r="K18" s="11" t="n"/>
+      <c r="K18" s="12" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
@@ -2858,7 +3159,7 @@
           <t>CL-2203</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
@@ -2868,17 +3169,17 @@
           <t>Crane failure, Rotterdam yard</t>
         </is>
       </c>
-      <c r="F19" s="18" t="n">
+      <c r="F19" s="19" t="n">
         <v>860</v>
       </c>
-      <c r="G19" s="24" t="n">
+      <c r="G19" s="25" t="n">
         <v>45203</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="12">
         <f>IF($C19="",ROW(),"")</f>
         <v>19</v>
       </c>
-      <c r="K19" s="11" t="n"/>
+      <c r="K19" s="12" t="n"/>
     </row>
     <row r="20">
       <c r="C20" s="4" t="inlineStr">
@@ -2886,7 +3187,7 @@
           <t>EV-302</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
@@ -2896,20 +3197,20 @@
           <t>Hailstorm, Po Valley</t>
         </is>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="19" t="n">
         <v>900</v>
       </c>
-      <c r="G20" s="24" t="n">
+      <c r="G20" s="25" t="n">
         <v>45465</v>
       </c>
-      <c r="H20" s="24" t="n">
+      <c r="H20" s="25" t="n">
         <v>45465</v>
       </c>
-      <c r="I20" s="18" t="n">
+      <c r="I20" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11">
+      <c r="J20" s="12" t="n"/>
+      <c r="K20" s="12">
         <f>IF($C20&lt;&gt;"",ROW(),"")</f>
         <v>20</v>
       </c>
@@ -2920,7 +3221,7 @@
           <t>EV-302</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
@@ -2930,20 +3231,20 @@
           <t>Hailstorm, Po Valley</t>
         </is>
       </c>
-      <c r="F21" s="18" t="n">
+      <c r="F21" s="19" t="n">
         <v>2600</v>
       </c>
-      <c r="G21" s="24" t="n">
+      <c r="G21" s="25" t="n">
         <v>45465</v>
       </c>
-      <c r="H21" s="24" t="n">
+      <c r="H21" s="25" t="n">
         <v>45465</v>
       </c>
-      <c r="I21" s="18" t="n">
+      <c r="I21" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="11">
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12">
         <f>IF($C21&lt;&gt;"",ROW(),"")</f>
         <v>21</v>
       </c>
@@ -2954,7 +3255,7 @@
           <t>CL-2204</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
@@ -2964,17 +3265,17 @@
           <t>Generator fire, Valencia plant</t>
         </is>
       </c>
-      <c r="F22" s="18" t="n">
+      <c r="F22" s="19" t="n">
         <v>1975</v>
       </c>
-      <c r="G22" s="24" t="n">
+      <c r="G22" s="25" t="n">
         <v>45503</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="12">
         <f>IF($C22="",ROW(),"")</f>
         <v>22</v>
       </c>
-      <c r="K22" s="11" t="n"/>
+      <c r="K22" s="12" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
@@ -2982,7 +3283,7 @@
           <t>CL-2205</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -2992,17 +3293,17 @@
           <t>Cable laying barge grounding, Kiel</t>
         </is>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="19" t="n">
         <v>1180</v>
       </c>
-      <c r="G23" s="24" t="n">
+      <c r="G23" s="25" t="n">
         <v>45789</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="12">
         <f>IF($C23="",ROW(),"")</f>
         <v>23</v>
       </c>
-      <c r="K23" s="11" t="n"/>
+      <c r="K23" s="12" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
@@ -3012,21 +3313,21 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Info_1 = J</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Info_2 = K</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>As at = 31.12.2025</t>
         </is>
@@ -3065,42 +3366,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Currency = USD</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Scale = 1,000</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Share basis = 100%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Exposure basis = Sum Insured</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Includes fac = yes</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Layered business = excluded</t>
         </is>
@@ -3114,34 +3415,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Section_1 = Engineering</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>As at_1 = 30.09.2025</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Risks</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>Sum insured</t>
         </is>
@@ -3153,27 +3454,27 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Header_1</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Number of Risks</t>
         </is>
       </c>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Exposure</t>
         </is>
@@ -3190,16 +3491,16 @@
           <t>0 – 1 000</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>1150</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>210</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="19" t="n">
         <v>96000</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="20">
         <f>ROW()</f>
         <v>12</v>
       </c>
@@ -3210,16 +3511,16 @@
           <t>1 001 – 5 000</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>2800</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <v>165</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <v>430000</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="20">
         <f>ROW()</f>
         <v>13</v>
       </c>
@@ -3230,16 +3531,16 @@
           <t>5 001 – 20 000</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>3450</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>78</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <v>780000</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="20">
         <f>ROW()</f>
         <v>14</v>
       </c>
@@ -3250,16 +3551,16 @@
           <t>&gt; 20 000</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>2900</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <v>940000</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="20">
         <f>ROW()</f>
         <v>15</v>
       </c>
@@ -3270,15 +3571,15 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="21">
         <f>SUM(E12:E15)</f>
         <v>10300</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="21">
         <f>SUM(F12:F15)</f>
         <v>480</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="21">
         <f>SUM(G12:G15)</f>
         <v>2246000</v>
       </c>
@@ -3289,7 +3590,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Info_1 = J</t>
         </is>

</xml_diff>